<commit_message>
Add Bandung variant of Buku Kolam Mitra; generalize builder by header names
The Kolam Mitra builder now locates columns by header text, reads the
wilayah list from the source dropdown, and treats Tingkat Risiko as
optional (the Bandung file has no risk column, so its dashboard swaps in
a Perjanjian Tertulis card and an Aktif vs Stop per Wilayah chart).
Regenerated the full-region workbook with the same script.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BxtPBXuWMP3d4NJHiNiQTv
</commit_message>
<xml_diff>
--- a/excel/Buku_Kolam_Mitra_Twenty_Swim.xlsx
+++ b/excel/Buku_Kolam_Mitra_Twenty_Swim.xlsx
@@ -3063,16 +3063,16 @@
           <t>Data kolam + info internal kerjasama. Sel kuning = ada catatan keluhan. Sel abu-abu muda = kolom yang masih perlu dilengkapi. Kolom dropdown tinggal pilih.</t>
         </is>
       </c>
-      <c r="L2" s="41" t="inlineStr">
+      <c r="M2" s="41" t="inlineStr">
         <is>
           <t>Terisi:</t>
         </is>
       </c>
-      <c r="M2" s="42">
+      <c r="N2" s="42">
         <f>COUNTA($B$5:$B$404)</f>
         <v/>
       </c>
-      <c r="N2" s="40" t="inlineStr">
+      <c r="O2" s="40" t="inlineStr">
         <is>
           <t>kolam</t>
         </is>
@@ -12251,11 +12251,11 @@
     <dataValidation sqref="K5:K404" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pilihan tidak valid" error="Silakan pilih dari daftar dropdown." type="list">
       <formula1>=Daftar!$I$2:$I$3</formula1>
     </dataValidation>
+    <dataValidation sqref="O5:O404" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pilihan tidak valid" error="Silakan pilih dari daftar dropdown." type="list">
+      <formula1>=Daftar!$M$2:$M$3</formula1>
+    </dataValidation>
     <dataValidation sqref="M5:M404" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pilihan tidak valid" error="Silakan pilih dari daftar dropdown." type="list">
       <formula1>=Daftar!$K$2:$K$4</formula1>
-    </dataValidation>
-    <dataValidation sqref="O5:O404" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pilihan tidak valid" error="Silakan pilih dari daftar dropdown." type="list">
-      <formula1>=Daftar!$M$2:$M$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13021,7 +13021,7 @@
       </c>
       <c r="G16" s="53" t="inlineStr">
         <is>
-          <t>Tertulis</t>
+          <t>Coach Gratis</t>
         </is>
       </c>
     </row>
@@ -13052,7 +13052,7 @@
         <v/>
       </c>
       <c r="G17" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A17,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A17,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>
@@ -13083,7 +13083,7 @@
         <v/>
       </c>
       <c r="G18" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A18,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A18,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
         <v/>
       </c>
       <c r="G19" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A19,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A19,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>
@@ -13145,7 +13145,7 @@
         <v/>
       </c>
       <c r="G20" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A20,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A20,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>
@@ -13176,7 +13176,7 @@
         <v/>
       </c>
       <c r="G21" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A21,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A21,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>
@@ -13207,7 +13207,7 @@
         <v/>
       </c>
       <c r="G22" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A22,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A22,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>
@@ -13238,7 +13238,7 @@
         <v/>
       </c>
       <c r="G23" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A23,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A23,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>
@@ -13269,7 +13269,7 @@
         <v/>
       </c>
       <c r="G24" s="54">
-        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A24,'Kolam Mitra'!$I$5:$I$404,"Tertulis")</f>
+        <f>COUNTIFS('Kolam Mitra'!$C$5:$C$404,$A24,'Kolam Mitra'!$J$5:$J$404,"Gratis")</f>
         <v/>
       </c>
     </row>

</xml_diff>